<commit_message>
Les 4 citations to PDF pages (Dummies Table 1-2 p. 41, 25 subgroups p. 244, Gauge R&R 20 % deck p. 61); F-interval bound 1.938
Dummies Table 1-2 sits on PDF p. 41 (raw S07 + merge, decision 3, Sigma sheet); decision 13's 'minimum of 25
subgroups' is on Dummies p. 244; 'Gauge R&R <= 20 % of tolerance' is on deck PDF p. 61. The Dummies F-interval
upper bound 0.5333 x 3.633 = 1.93765 rounds to 1.938 (README, test reason). Oracle unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/build/bb_toolkit.xlsx
+++ b/build/bb_toolkit.xlsx
@@ -20898,7 +20898,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>source/course/Les 4/2026 Lean - Six Sigma v13 - Capabiliteit - SPC.pdf p. 20-21, 37-40; Six Sigma For Dummies.pdf p. 42, 147-161; Six-Sigma Mikel Harry - Richard Schroeder.pdf p. 3-5; 20260521_van volsem.pdf p. 7</t>
+          <t>source/course/Les 4/2026 Lean - Six Sigma v13 - Capabiliteit - SPC.pdf p. 20-21, 37-40; Six Sigma For Dummies.pdf p. 41, 147-161; Six-Sigma Mikel Harry - Richard Schroeder.pdf p. 3-5; 20260521_van volsem.pdf p. 7</t>
         </is>
       </c>
     </row>
@@ -21193,7 +21193,7 @@
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>deck p. 21; Dummies p. 42, 160; Van Volsem p. 7: 6 -&gt; 3.4</t>
+          <t>deck p. 21; Dummies p. 41, 160; Van Volsem p. 7: 6 -&gt; 3.4</t>
         </is>
       </c>
     </row>
@@ -41091,7 +41091,7 @@
     <row r="86">
       <c r="A86" s="8" t="inlineStr">
         <is>
-          <t>Other course thresholds: 'Gauge R&amp;R ≤ 20 % of tolerance' (deck Les 4 p. 60); σ²_measure / σ²_observed ≤ 0.1 good, 0.1-0.3 marginal, ≥ 0.3 unacceptable (Dummies p. 178).</t>
+          <t>Other course thresholds: 'Gauge R&amp;R ≤ 20 % of tolerance' (deck Les 4 p. 61); σ²_measure / σ²_observed ≤ 0.1 good, 0.1-0.3 marginal, ≥ 0.3 unacceptable (Dummies p. 178).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Workbook header block and README in Dutch; guide links to documents and cross-references open in a new tab
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/build/bb_toolkit.xlsx
+++ b/build/bb_toolkit.xlsx
@@ -1235,7 +1235,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Course source</t>
+          <t>Bron in de cursus</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Convention used</t>
+          <t>Gebruikte conventie</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -1264,31 +1264,31 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>VERIFIED: tested against course worked examples S06-WE01, S06-WE02, S06-WE04, S06-WE07, S06-WE08, S06-WE12, S06-WE13; a few printed values on deck p. 46 and 50 disagree with the computation (listed in build/README.md)</t>
+          <t>GEVERIFIEERD (VERIFIED): tested against course worked examples S06-WE01, S06-WE02, S06-WE04, S06-WE07, S06-WE08, S06-WE12, S06-WE13; a few printed values on deck p. 46 and 50 disagree with the computation (listed in build/README.md)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Legend</t>
+          <t>Legende</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Yellow cell = type your input here.  Green cell = result, do not type.  Orange cell (Tables) = disagrees with another printed source.</t>
+          <t>Gele cel = vul hier in (invoer).  Groene cel = resultaat, niet overtypen.  Oranje cel (Tabellen) = verschilt van een andere gedrukte bron.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Controle</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>If a green cell shows nothing, an input it needs is still empty.</t>
+          <t>Blijft een groene cel leeg, dan ontbreekt nog een invoer die ze nodig heeft.</t>
         </is>
       </c>
     </row>
@@ -2198,7 +2198,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Course source</t>
+          <t>Bron in de cursus</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -2210,7 +2210,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Convention used</t>
+          <t>Gebruikte conventie</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -2227,31 +2227,31 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>VERIFIED: tested against course worked examples S03-WE06, S03-WE07, S03-WE20, S03-WE21, S04-WE12, S04-WE16, S04-WE18</t>
+          <t>GEVERIFIEERD (VERIFIED): tested against course worked examples S03-WE06, S03-WE07, S03-WE20, S03-WE21, S04-WE12, S04-WE16, S04-WE18</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Legend</t>
+          <t>Legende</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Yellow cell = type your input here.  Green cell = result, do not type.  Orange cell (Tables) = disagrees with another printed source.</t>
+          <t>Gele cel = vul hier in (invoer).  Groene cel = resultaat, niet overtypen.  Oranje cel (Tabellen) = verschilt van een andere gedrukte bron.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Controle</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>If a green cell shows nothing, an input it needs is still empty.</t>
+          <t>Blijft een groene cel leeg, dan ontbreekt nog een invoer die ze nodig heeft.</t>
         </is>
       </c>
     </row>
@@ -3861,7 +3861,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Course source</t>
+          <t>Bron in de cursus</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -3873,7 +3873,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Convention used</t>
+          <t>Gebruikte conventie</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -3890,31 +3890,31 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>VERIFIED: tested against course worked examples S05-WE01, S05-WE02, S05-WE05 to S05-WE09, S05-WE17, S05-WE18, S08-WE16; printed values that disagree are listed in build/README.md</t>
+          <t>GEVERIFIEERD (VERIFIED): tested against course worked examples S05-WE01, S05-WE02, S05-WE05 to S05-WE09, S05-WE17, S05-WE18, S08-WE16; printed values that disagree are listed in build/README.md</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Legend</t>
+          <t>Legende</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Yellow cell = type your input here.  Green cell = result, do not type.  Orange cell (Tables) = disagrees with another printed source.</t>
+          <t>Gele cel = vul hier in (invoer).  Groene cel = resultaat, niet overtypen.  Oranje cel (Tabellen) = verschilt van een andere gedrukte bron.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Controle</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>If a green cell shows nothing, an input it needs is still empty.</t>
+          <t>Blijft een groene cel leeg, dan ontbreekt nog een invoer die ze nodig heeft.</t>
         </is>
       </c>
     </row>
@@ -13487,7 +13487,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Course source</t>
+          <t>Bron in de cursus</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -13499,7 +13499,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Convention used</t>
+          <t>Gebruikte conventie</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -13516,31 +13516,31 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>VERIFIED: transcriptions of both scanned tables double-checked cell by cell; values compared with their mathematical definitions in tests/test_constants.py</t>
+          <t>GEVERIFIEERD (VERIFIED): transcriptions of both scanned tables double-checked cell by cell; values compared with their mathematical definitions in tests/test_constants.py</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Legend</t>
+          <t>Legende</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Yellow cell = type your input here.  Green cell = result, do not type.  Orange cell (Tables) = disagrees with another printed source.</t>
+          <t>Gele cel = vul hier in (invoer).  Groene cel = resultaat, niet overtypen.  Oranje cel (Tabellen) = verschilt van een andere gedrukte bron.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Controle</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>If a green cell shows nothing, an input it needs is still empty.</t>
+          <t>Blijft een groene cel leeg, dan ontbreekt nog een invoer die ze nodig heeft.</t>
         </is>
       </c>
     </row>
@@ -20314,7 +20314,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Course source</t>
+          <t>Bron in de cursus</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -20326,7 +20326,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Convention used</t>
+          <t>Gebruikte conventie</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -20343,31 +20343,31 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>VERIFIED: tested against course worked examples S06-WE09 (NORM.INV / NORM.VERD workbook) and S06-WE10 (deck p. 19 notes), the 68-95-99.7 rule (deck p. 19) and the course Z table</t>
+          <t>GEVERIFIEERD (VERIFIED): tested against course worked examples S06-WE09 (NORM.INV / NORM.VERD workbook) and S06-WE10 (deck p. 19 notes), the 68-95-99.7 rule (deck p. 19) and the course Z table</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Legend</t>
+          <t>Legende</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Yellow cell = type your input here.  Green cell = result, do not type.  Orange cell (Tables) = disagrees with another printed source.</t>
+          <t>Gele cel = vul hier in (invoer).  Groene cel = resultaat, niet overtypen.  Oranje cel (Tabellen) = verschilt van een andere gedrukte bron.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Controle</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>If a green cell shows nothing, an input it needs is still empty.</t>
+          <t>Blijft een groene cel leeg, dan ontbreekt nog een invoer die ze nodig heeft.</t>
         </is>
       </c>
     </row>
@@ -20893,7 +20893,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Course source</t>
+          <t>Bron in de cursus</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -20905,7 +20905,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Convention used</t>
+          <t>Gebruikte conventie</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -20922,31 +20922,31 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>VERIFIED: tested against course worked examples S07-WE01, S08-WE01 to S08-WE08, S09-WE01, S09-WE03 to S09-WE06 and the course sigma tables; a few printed values disagree (listed in build/README.md)</t>
+          <t>GEVERIFIEERD (VERIFIED): tested against course worked examples S07-WE01, S08-WE01 to S08-WE08, S09-WE01, S09-WE03 to S09-WE06 and the course sigma tables; a few printed values disagree (listed in build/README.md)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Legend</t>
+          <t>Legende</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Yellow cell = type your input here.  Green cell = result, do not type.  Orange cell (Tables) = disagrees with another printed source.</t>
+          <t>Gele cel = vul hier in (invoer).  Groene cel = resultaat, niet overtypen.  Oranje cel (Tabellen) = verschilt van een andere gedrukte bron.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Controle</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>If a green cell shows nothing, an input it needs is still empty.</t>
+          <t>Blijft een groene cel leeg, dan ontbreekt nog een invoer die ze nodig heeft.</t>
         </is>
       </c>
     </row>
@@ -21774,7 +21774,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Course source</t>
+          <t>Bron in de cursus</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -21786,7 +21786,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Convention used</t>
+          <t>Gebruikte conventie</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -21803,31 +21803,31 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>VERIFIED: tested against course worked examples S03-WE03, S03-WE05, S08-WE10 and the Dummies χ² and F tables (p. 194, 196); the Dummies F-interval example S08-WE11 disagrees (build/README.md)</t>
+          <t>GEVERIFIEERD (VERIFIED): tested against course worked examples S03-WE03, S03-WE05, S08-WE10 and the Dummies χ² and F tables (p. 194, 196); the Dummies F-interval example S08-WE11 disagrees (build/README.md)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Legend</t>
+          <t>Legende</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Yellow cell = type your input here.  Green cell = result, do not type.  Orange cell (Tables) = disagrees with another printed source.</t>
+          <t>Gele cel = vul hier in (invoer).  Groene cel = resultaat, niet overtypen.  Oranje cel (Tabellen) = verschilt van een andere gedrukte bron.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Controle</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>If a green cell shows nothing, an input it needs is still empty.</t>
+          <t>Blijft een groene cel leeg, dan ontbreekt nog een invoer die ze nodig heeft.</t>
         </is>
       </c>
     </row>
@@ -24542,7 +24542,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Course source</t>
+          <t>Bron in de cursus</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -24554,7 +24554,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Convention used</t>
+          <t>Gebruikte conventie</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -24571,31 +24571,31 @@
       </c>
       <c r="B4" s="30" t="inlineStr">
         <is>
-          <t>UNVERIFIED: no course worked example prints these metrics; checked against an independent computation and by the stats-auditor (build/README.md)</t>
+          <t>NIET GEVERIFIEERD (UNVERIFIED): no course worked example prints these metrics; checked against an independent computation and by the stats-auditor (build/README.md)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Legend</t>
+          <t>Legende</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Yellow cell = type your input here.  Green cell = result, do not type.  Orange cell (Tables) = disagrees with another printed source.</t>
+          <t>Gele cel = vul hier in (invoer).  Groene cel = resultaat, niet overtypen.  Oranje cel (Tabellen) = verschilt van een andere gedrukte bron.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Controle</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>If a green cell shows nothing, an input it needs is still empty.</t>
+          <t>Blijft een groene cel leeg, dan ontbreekt nog een invoer die ze nodig heeft.</t>
         </is>
       </c>
     </row>
@@ -25644,7 +25644,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Course source</t>
+          <t>Bron in de cursus</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -25656,7 +25656,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Convention used</t>
+          <t>Gebruikte conventie</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -25673,31 +25673,31 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>VERIFIED: binomial and hypergeometric blocks tested against course worked examples S04-WE02, S03-WE19, S03-WE21, the Poisson block against S02-WE09; Bernoulli, Poisson, exponential and uniform use standard definitions not printed in the course (decision 20; audited)</t>
+          <t>GEVERIFIEERD (VERIFIED): binomial and hypergeometric blocks tested against course worked examples S04-WE02, S03-WE19, S03-WE21, the Poisson block against S02-WE09; Bernoulli, Poisson, exponential and uniform use standard definitions not printed in the course (decision 20; audited)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Legend</t>
+          <t>Legende</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Yellow cell = type your input here.  Green cell = result, do not type.  Orange cell (Tables) = disagrees with another printed source.</t>
+          <t>Gele cel = vul hier in (invoer).  Groene cel = resultaat, niet overtypen.  Oranje cel (Tabellen) = verschilt van een andere gedrukte bron.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Controle</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>If a green cell shows nothing, an input it needs is still empty.</t>
+          <t>Blijft een groene cel leeg, dan ontbreekt nog een invoer die ze nodig heeft.</t>
         </is>
       </c>
     </row>
@@ -26282,7 +26282,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Course source</t>
+          <t>Bron in de cursus</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -26294,7 +26294,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Convention used</t>
+          <t>Gebruikte conventie</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -26311,31 +26311,31 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>VERIFIED: tested against course worked examples S03-WE01, S03-WE02, S03-WE04, S03-WE10, S03-WE13, S03-WE14, S03-WE15, S08-WE12, S08-WE13</t>
+          <t>GEVERIFIEERD (VERIFIED): tested against course worked examples S03-WE01, S03-WE02, S03-WE04, S03-WE10, S03-WE13, S03-WE14, S03-WE15, S08-WE12, S08-WE13</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Legend</t>
+          <t>Legende</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Yellow cell = type your input here.  Green cell = result, do not type.  Orange cell (Tables) = disagrees with another printed source.</t>
+          <t>Gele cel = vul hier in (invoer).  Groene cel = resultaat, niet overtypen.  Oranje cel (Tabellen) = verschilt van een andere gedrukte bron.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Controle</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>If a green cell shows nothing, an input it needs is still empty.</t>
+          <t>Blijft een groene cel leeg, dan ontbreekt nog een invoer die ze nodig heeft.</t>
         </is>
       </c>
     </row>
@@ -32048,7 +32048,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Course source</t>
+          <t>Bron in de cursus</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -32060,7 +32060,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Convention used</t>
+          <t>Gebruikte conventie</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -32077,31 +32077,31 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>VERIFIED: tested against course worked examples S06-WE03, S06-WE05, S06-WE06, S08-WE18, S08-WE21, S10-WE04a, S10-WE04b; a few printed values disagree (build/README.md)</t>
+          <t>GEVERIFIEERD (VERIFIED): tested against course worked examples S06-WE03, S06-WE05, S06-WE06, S08-WE18, S08-WE21, S10-WE04a, S10-WE04b; a few printed values disagree (build/README.md)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Legend</t>
+          <t>Legende</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Yellow cell = type your input here.  Green cell = result, do not type.  Orange cell (Tables) = disagrees with another printed source.</t>
+          <t>Gele cel = vul hier in (invoer).  Groene cel = resultaat, niet overtypen.  Oranje cel (Tabellen) = verschilt van een andere gedrukte bron.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Controle</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>If a green cell shows nothing, an input it needs is still empty.</t>
+          <t>Blijft een groene cel leeg, dan ontbreekt nog een invoer die ze nodig heeft.</t>
         </is>
       </c>
     </row>
@@ -39611,7 +39611,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Course source</t>
+          <t>Bron in de cursus</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -39623,7 +39623,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Convention used</t>
+          <t>Gebruikte conventie</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -39640,31 +39640,31 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>VERIFIED: tested against course worked examples S10-WE02 (ANOVA) and S10-WE03 (average and range) on the course's own study data</t>
+          <t>GEVERIFIEERD (VERIFIED): tested against course worked examples S10-WE02 (ANOVA) and S10-WE03 (average and range) on the course's own study data</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Legend</t>
+          <t>Legende</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Yellow cell = type your input here.  Green cell = result, do not type.  Orange cell (Tables) = disagrees with another printed source.</t>
+          <t>Gele cel = vul hier in (invoer).  Groene cel = resultaat, niet overtypen.  Oranje cel (Tabellen) = verschilt van een andere gedrukte bron.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Controle</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>If a green cell shows nothing, an input it needs is still empty.</t>
+          <t>Blijft een groene cel leeg, dan ontbreekt nog een invoer die ze nodig heeft.</t>
         </is>
       </c>
     </row>

</xml_diff>